<commit_message>
feature/fsel-4307: Export file Report PlacementTest Event
</commit_message>
<xml_diff>
--- a/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ExportExcelTemplates/ReportPTEvent.xlsx
+++ b/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ExportExcelTemplates/ReportPTEvent.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Backend\Fsel_src\Services\Fsel.Course\Fsel.Course.Lms.Api\Resources\ExportExcelTemplates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B9669213-FE99-4B83-8D2F-891D10A0527D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{824EFF17-D9D9-4FFC-BF21-3482DEC91DB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{115BFFB9-1295-4567-8593-4DA8B1A07CE0}"/>
+    <workbookView xWindow="-28800" yWindow="1890" windowWidth="29730" windowHeight="11295" xr2:uid="{115BFFB9-1295-4567-8593-4DA8B1A07CE0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -96,7 +96,7 @@
     <t>C1</t>
   </si>
   <si>
-    <t>{0} SỐ LIỆU ĐĂNG KÝ &amp; KẾT QUẢ ĐÁNH GIÁ NĂNG LỰC ĐẦU VÀO TIẾNG ANH TRÊN HỆ THỐNG - PLACEMENT TEST (PT)</t>
+    <t>[{0}] SỐ LIỆU ĐĂNG KÝ &amp; KẾT QUẢ ĐÁNH GIÁ NĂNG LỰC ĐẦU VÀO TIẾNG ANH TRÊN HỆ THỐNG - PLACEMENT TEST (PT)</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
feature/fsel-4528: Update Report File PT
</commit_message>
<xml_diff>
--- a/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ExportExcelTemplates/ReportPTEvent.xlsx
+++ b/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ExportExcelTemplates/ReportPTEvent.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Backend\Fsel_src\Services\Fsel.Course\Fsel.Course.Lms.Api\Resources\ExportExcelTemplates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Backend\fsel_src\Services\Fsel.Course\Fsel.Course.Lms.Api\Resources\ExportExcelTemplates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{824EFF17-D9D9-4FFC-BF21-3482DEC91DB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ADE3C09-4E91-4C8E-A53A-0D997A489E6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28800" yWindow="1890" windowWidth="29730" windowHeight="11295" xr2:uid="{115BFFB9-1295-4567-8593-4DA8B1A07CE0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{115BFFB9-1295-4567-8593-4DA8B1A07CE0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="25">
   <si>
     <t>TEMPLATE BÁO CÁO SỰ KIỆN SỞ HN</t>
   </si>
@@ -66,9 +66,6 @@
     <t>Tỷ lệ HS</t>
   </si>
   <si>
-    <t>Hoàn thành PT/Đăng ký TK</t>
-  </si>
-  <si>
     <t>Trình độ PT trên hệ thống FSEL*</t>
   </si>
   <si>
@@ -97,6 +94,12 @@
   </si>
   <si>
     <t>[{0}] SỐ LIỆU ĐĂNG KÝ &amp; KẾT QUẢ ĐÁNH GIÁ NĂNG LỰC ĐẦU VÀO TIẾNG ANH TRÊN HỆ THỐNG - PLACEMENT TEST (PT)</t>
+  </si>
+  <si>
+    <t>xác thực thành công</t>
+  </si>
+  <si>
+    <t>Hoàn thành PT/Xác thực thành công</t>
   </si>
 </sst>
 </file>
@@ -687,10 +690,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBE1EA8C-D46E-4A59-B00F-A34792F32A0D}">
-  <dimension ref="A1:T8"/>
+  <dimension ref="A1:V8"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="8" max="8" width="9.125" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="10" max="10" width="16.25" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -713,8 +721,10 @@
       <c r="R1" s="2"/>
       <c r="S1" s="2"/>
       <c r="T1" s="2"/>
+      <c r="U1" s="2"/>
+      <c r="V1" s="2"/>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
       <c r="C2" s="4"/>
@@ -735,8 +745,10 @@
       <c r="R2" s="4"/>
       <c r="S2" s="4"/>
       <c r="T2" s="4"/>
+      <c r="U2" s="4"/>
+      <c r="V2" s="4"/>
     </row>
-    <row r="3" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>1</v>
       </c>
@@ -759,8 +771,10 @@
       <c r="R3" s="4"/>
       <c r="S3" s="4"/>
       <c r="T3" s="4"/>
+      <c r="U3" s="4"/>
+      <c r="V3" s="4"/>
     </row>
-    <row r="4" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
       <c r="B4" s="3"/>
       <c r="C4" s="4"/>
@@ -781,10 +795,12 @@
       <c r="R4" s="4"/>
       <c r="S4" s="4"/>
       <c r="T4" s="4"/>
+      <c r="U4" s="4"/>
+      <c r="V4" s="4"/>
     </row>
-    <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="11"/>
@@ -805,8 +821,10 @@
       <c r="R5" s="11"/>
       <c r="S5" s="11"/>
       <c r="T5" s="11"/>
+      <c r="U5" s="11"/>
+      <c r="V5" s="11"/>
     </row>
-    <row r="6" spans="1:20" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:22" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
         <v>2</v>
       </c>
@@ -831,11 +849,15 @@
       <c r="H6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="J6" s="16"/>
-      <c r="K6" s="16"/>
+      <c r="I6" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="K6" s="15" t="s">
+        <v>13</v>
+      </c>
       <c r="L6" s="16"/>
       <c r="M6" s="16"/>
       <c r="N6" s="16"/>
@@ -844,9 +866,11 @@
       <c r="Q6" s="16"/>
       <c r="R6" s="16"/>
       <c r="S6" s="16"/>
-      <c r="T6" s="17"/>
+      <c r="T6" s="16"/>
+      <c r="U6" s="16"/>
+      <c r="V6" s="17"/>
     </row>
-    <row r="7" spans="1:20" ht="51" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:22" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A7" s="13"/>
       <c r="B7" s="13"/>
       <c r="C7" s="7" t="s">
@@ -862,16 +886,20 @@
         <v>10</v>
       </c>
       <c r="G7" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="I7" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="I7" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="J7" s="19"/>
-      <c r="K7" s="19"/>
+      <c r="J7" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K7" s="18" t="s">
+        <v>14</v>
+      </c>
       <c r="L7" s="19"/>
       <c r="M7" s="19"/>
       <c r="N7" s="19"/>
@@ -880,9 +908,11 @@
       <c r="Q7" s="19"/>
       <c r="R7" s="19"/>
       <c r="S7" s="19"/>
-      <c r="T7" s="20"/>
+      <c r="T7" s="19"/>
+      <c r="U7" s="19"/>
+      <c r="V7" s="20"/>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A8" s="14"/>
       <c r="B8" s="14"/>
       <c r="C8" s="8"/>
@@ -891,50 +921,52 @@
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
       <c r="H8" s="8"/>
-      <c r="I8" s="9" t="s">
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="L8" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="J8" s="9" t="s">
+      <c r="M8" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="K8" s="9" t="s">
+      <c r="N8" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="O8" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="L8" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="M8" s="9" t="s">
+      <c r="P8" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q8" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="N8" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="O8" s="9" t="s">
+      <c r="R8" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="S8" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="P8" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q8" s="9" t="s">
+      <c r="T8" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="U8" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="R8" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="S8" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="T8" s="9" t="s">
-        <v>17</v>
+      <c r="V8" s="9" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A5:T5"/>
+    <mergeCell ref="A5:V5"/>
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="B6:B8"/>
-    <mergeCell ref="I6:T6"/>
-    <mergeCell ref="I7:T7"/>
+    <mergeCell ref="K6:V6"/>
+    <mergeCell ref="K7:V7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feature/fsel-4528: Update Event Report PT
</commit_message>
<xml_diff>
--- a/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ExportExcelTemplates/ReportPTEvent.xlsx
+++ b/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ExportExcelTemplates/ReportPTEvent.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Backend\fsel_src\Services\Fsel.Course\Fsel.Course.Lms.Api\Resources\ExportExcelTemplates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ADE3C09-4E91-4C8E-A53A-0D997A489E6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EE87C76-8D3C-4AF5-A177-BC427BB02106}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{115BFFB9-1295-4567-8593-4DA8B1A07CE0}"/>
+    <workbookView xWindow="-28920" yWindow="-135" windowWidth="29040" windowHeight="15720" xr2:uid="{115BFFB9-1295-4567-8593-4DA8B1A07CE0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="26">
   <si>
     <t>TEMPLATE BÁO CÁO SỰ KIỆN SỞ HN</t>
   </si>
@@ -100,6 +100,9 @@
   </si>
   <si>
     <t>Hoàn thành PT/Xác thực thành công</t>
+  </si>
+  <si>
+    <t>Đang làm bài PT</t>
   </si>
 </sst>
 </file>
@@ -690,15 +693,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBE1EA8C-D46E-4A59-B00F-A34792F32A0D}">
-  <dimension ref="A1:V8"/>
+  <dimension ref="A1:W8"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="8" max="8" width="9.125" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="16.25" customWidth="1"/>
+    <col min="8" max="9" width="9.125" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="16.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -723,8 +726,9 @@
       <c r="T1" s="2"/>
       <c r="U1" s="2"/>
       <c r="V1" s="2"/>
+      <c r="W1" s="2"/>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
       <c r="C2" s="4"/>
@@ -747,8 +751,9 @@
       <c r="T2" s="4"/>
       <c r="U2" s="4"/>
       <c r="V2" s="4"/>
+      <c r="W2" s="4"/>
     </row>
-    <row r="3" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>1</v>
       </c>
@@ -773,8 +778,9 @@
       <c r="T3" s="4"/>
       <c r="U3" s="4"/>
       <c r="V3" s="4"/>
+      <c r="W3" s="4"/>
     </row>
-    <row r="4" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
       <c r="B4" s="3"/>
       <c r="C4" s="4"/>
@@ -797,8 +803,9 @@
       <c r="T4" s="4"/>
       <c r="U4" s="4"/>
       <c r="V4" s="4"/>
+      <c r="W4" s="4"/>
     </row>
-    <row r="5" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="10" t="s">
         <v>22</v>
       </c>
@@ -823,8 +830,9 @@
       <c r="T5" s="11"/>
       <c r="U5" s="11"/>
       <c r="V5" s="11"/>
+      <c r="W5" s="11"/>
     </row>
-    <row r="6" spans="1:22" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:23" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
         <v>2</v>
       </c>
@@ -853,12 +861,14 @@
         <v>9</v>
       </c>
       <c r="J6" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="K6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="K6" s="15" t="s">
+      <c r="L6" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="L6" s="16"/>
       <c r="M6" s="16"/>
       <c r="N6" s="16"/>
       <c r="O6" s="16"/>
@@ -868,9 +878,10 @@
       <c r="S6" s="16"/>
       <c r="T6" s="16"/>
       <c r="U6" s="16"/>
-      <c r="V6" s="17"/>
+      <c r="V6" s="16"/>
+      <c r="W6" s="17"/>
     </row>
-    <row r="7" spans="1:22" ht="76.5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:23" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A7" s="13"/>
       <c r="B7" s="13"/>
       <c r="C7" s="7" t="s">
@@ -892,15 +903,17 @@
         <v>23</v>
       </c>
       <c r="I7" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="J7" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="J7" s="7" t="s">
+      <c r="K7" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="K7" s="18" t="s">
+      <c r="L7" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="L7" s="19"/>
       <c r="M7" s="19"/>
       <c r="N7" s="19"/>
       <c r="O7" s="19"/>
@@ -910,9 +923,10 @@
       <c r="S7" s="19"/>
       <c r="T7" s="19"/>
       <c r="U7" s="19"/>
-      <c r="V7" s="20"/>
+      <c r="V7" s="19"/>
+      <c r="W7" s="20"/>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A8" s="14"/>
       <c r="B8" s="14"/>
       <c r="C8" s="8"/>
@@ -923,50 +937,51 @@
       <c r="H8" s="8"/>
       <c r="I8" s="8"/>
       <c r="J8" s="8"/>
-      <c r="K8" s="9" t="s">
+      <c r="K8" s="8"/>
+      <c r="L8" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="L8" s="9" t="s">
+      <c r="M8" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="M8" s="9" t="s">
+      <c r="N8" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="N8" s="9" t="s">
+      <c r="O8" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="O8" s="9" t="s">
+      <c r="P8" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="P8" s="9" t="s">
+      <c r="Q8" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="Q8" s="9" t="s">
+      <c r="R8" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="R8" s="9" t="s">
+      <c r="S8" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="S8" s="9" t="s">
+      <c r="T8" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="T8" s="9" t="s">
+      <c r="U8" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="U8" s="9" t="s">
+      <c r="V8" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="V8" s="9" t="s">
+      <c r="W8" s="9" t="s">
         <v>16</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A5:V5"/>
+    <mergeCell ref="A5:W5"/>
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="B6:B8"/>
-    <mergeCell ref="K6:V6"/>
-    <mergeCell ref="K7:V7"/>
+    <mergeCell ref="L6:W6"/>
+    <mergeCell ref="L7:W7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>